<commit_message>
Split into two Lead Gen Forms for clean two-scenario attribution
Per Fabien's decision to build two Make.com scenarios (one per ad):
LinkedIn's Lead Gen Form response carries no ad-level field, so two
scenarios watching one shared form couldn't reliably split by
concept. Changed the plan to two identical forms, one per ad, each
watched by its own scenario, each writing a static Concept value into
the sheet. Updated the tracker's Make.com Setup tab, the brief's Lead
Gen Form section, and the sequencing checklist to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014zdMVC2PGgF2M5N7pSgc3d
</commit_message>
<xml_diff>
--- a/halo-growth-hvac/hvac-qualified-lead-tracker.xlsx
+++ b/halo-growth-hvac/hvac-qualified-lead-tracker.xlsx
@@ -148,7 +148,7 @@
     <t xml:space="preserve">Leads — one row per HVAC business submission</t>
   </si>
   <si>
-    <t xml:space="preserve">Populated automatically by Make.com once connected (see Make.com Setup tab), or paste in manually from a LinkedIn Campaign Manager CSV export meanwhile. Concept must be A or C exactly to match Campaign Summary's formulas.</t>
+    <t xml:space="preserve">Populated automatically by two Make.com scenarios (one per ad, see Make.com Setup tab), or paste in manually from a LinkedIn Campaign Manager CSV export meanwhile.</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
@@ -211,31 +211,31 @@
     <t xml:space="preserve">Connecting LinkedIn Lead Gen Forms to this sheet via Make.com</t>
   </si>
   <si>
-    <t xml:space="preserve">I have no LinkedIn or Make.com access in this session, so this hasn't been built or tested. Steps below are the standard, documented way to do this in Make; verify against Make's actual current UI as you go.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. This file needs to be a Google Sheet, not a local .xlsx, for Make to write into it live. Upload/import this file into Google Sheets first (File &gt; Import &gt; Upload, replace spreadsheet, keeps the formulas and formatting).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. In Make.com, create a new Scenario. Add a trigger module: search for 'LinkedIn Lead Gen Ads', choose 'Watch Leads' (or the equivalent new-lead trigger). Connect your LinkedIn Ads account (needs admin access on the ad account running this campaign).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Select the specific Lead Gen Form built for this campaign ('HVAC 5-Opportunity Trial', per CLAUDE_BROWSER_LINKEDIN_BRIEF.md).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. Add an action module: 'Google Sheets' -&gt; 'Add a Row'. Connect the Google account that owns the imported sheet from step 1, select this spreadsheet, and the 'Leads' tab.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Map LinkedIn's form fields to this sheet's columns: Date -&gt; use Make's 'now' function, Company -&gt; Company, Contact name -&gt; Contact name, Email -&gt; Email, Phone -&gt; Phone. Concept (A/C), Qualified, and everything from 'Sales conversation held' onward are NOT in the LinkedIn form, leave those blank for manual entry after each lead comes in.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Run the scenario once manually with a real or sample submission before scheduling it, confirm a row actually appears in the right columns.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. Turn scheduling on (Make can run this near-instantly or on an interval). From this point, every new form submission should append a row automatically.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which column is 'Concept (A/C)' matched to which ad? Make can't infer this from the form alone unless you build two separate scenarios (one per ad) or add a hidden form field per ad. Worth deciding before wiring this up, not after.</t>
+    <t xml:space="preserve">Decided: two separate Lead Gen Forms (one per ad), each with its own Make scenario, so Concept A/C attribution is automatic rather than guessed. I have no LinkedIn or Make.com access in this session, so this hasn't been built or tested; verify against Make's actual current UI as you go.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0. In Campaign Manager, build two Lead Gen Forms with identical content (same fields, headline, supporting copy, confirmation message from CLAUDE_BROWSER_LINKEDIN_BRIEF.md), one attached to Ad 1 (Concept A) and one to Ad 2 (Concept C). This replaces the earlier one-shared-form plan, needed so each Make scenario can watch its own form and know which concept it belongs to.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Import this file into Google Sheets first (File &gt; Import &gt; Upload, replace spreadsheet), Make writes to a live Google Sheet, not a local .xlsx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Build Scenario 1 (Concept A): trigger module 'LinkedIn Lead Gen Ads' -&gt; 'Watch Leads', connect the LinkedIn Ads account, select the Concept A form specifically.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Action module: 'Google Sheets' -&gt; 'Add a Row', target this spreadsheet's 'Leads' tab. Map Date -&gt; now(), Company/Contact name/Email/Phone -&gt; the matching form fields, and set the 'Concept (A/C)' column to a static value: A.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Build Scenario 2 (Concept C): identical to Scenario 1, but watching the Concept C form, and the 'Concept (A/C)' column set to a static value: C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Qualified, Sales conversation held, Trial purchased, Repeat purchase, and Revenue are not in LinkedIn's form, leave those blank in both scenarios for manual entry after each lead comes in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Run each scenario once manually with a test submission before scheduling, confirm the row lands in the right columns with the correct Concept value.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Turn both scenarios on. From this point, every new form submission on either ad should append a correctly-attributed row automatically.</t>
   </si>
 </sst>
 </file>
@@ -394,7 +394,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -489,10 +489,6 @@
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -2697,7 +2693,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="1" style="0" width="30"/>
@@ -2773,13 +2769,13 @@
       <c r="C10" s="23"/>
       <c r="D10" s="23"/>
     </row>
-    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
+    <row r="11" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -2792,7 +2788,7 @@
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A11:D11"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>